<commit_message>
Standardize validation report outputs, and define true and false values
</commit_message>
<xml_diff>
--- a/data/exports/synergi_validation_results.xlsx
+++ b/data/exports/synergi_validation_results.xlsx
@@ -539,7 +539,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BS1"/>
+  <dimension ref="A1:BX1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -896,6 +896,31 @@
       <c r="BS1" t="inlineStr">
         <is>
           <t>IsFed</t>
+        </is>
+      </c>
+      <c r="BT1" t="inlineStr">
+        <is>
+          <t>RuleID</t>
+        </is>
+      </c>
+      <c r="BU1" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="BV1" t="inlineStr">
+        <is>
+          <t>Severity</t>
+        </is>
+      </c>
+      <c r="BW1" t="inlineStr">
+        <is>
+          <t>Issue</t>
+        </is>
+      </c>
+      <c r="BX1" t="inlineStr">
+        <is>
+          <t>RecommendedAction</t>
         </is>
       </c>
     </row>
@@ -7724,7 +7749,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AO1"/>
+  <dimension ref="A1:AU1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7931,6 +7956,36 @@
       <c r="AO1" t="inlineStr">
         <is>
           <t>VfiMinResSec</t>
+        </is>
+      </c>
+      <c r="AP1" t="inlineStr">
+        <is>
+          <t>RuleID</t>
+        </is>
+      </c>
+      <c r="AQ1" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="AR1" t="inlineStr">
+        <is>
+          <t>Severity</t>
+        </is>
+      </c>
+      <c r="AS1" t="inlineStr">
+        <is>
+          <t>Issue</t>
+        </is>
+      </c>
+      <c r="AT1" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="AU1" t="inlineStr">
+        <is>
+          <t>RecommendedAction</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
added rules.py and removed hardcoded VR#'s from all files
</commit_message>
<xml_diff>
--- a/data/exports/synergi_validation_results.xlsx
+++ b/data/exports/synergi_validation_results.xlsx
@@ -539,7 +539,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BX1"/>
+  <dimension ref="A1:BZ1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -915,10 +915,20 @@
       </c>
       <c r="BW1" t="inlineStr">
         <is>
+          <t>ElementType</t>
+        </is>
+      </c>
+      <c r="BX1" t="inlineStr">
+        <is>
+          <t>ElementID</t>
+        </is>
+      </c>
+      <c r="BY1" t="inlineStr">
+        <is>
           <t>Issue</t>
         </is>
       </c>
-      <c r="BX1" t="inlineStr">
+      <c r="BZ1" t="inlineStr">
         <is>
           <t>RecommendedAction</t>
         </is>
@@ -1358,7 +1368,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Conductor height sign does not match the inferred underground or overhead conductor type.</t>
+          <t>Section has negative height or elevation value.</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -1590,17 +1600,17 @@
       </c>
       <c r="BT2" t="inlineStr">
         <is>
-          <t>UG Conductor Height Should Be Negative</t>
+          <t>Section at negative height</t>
         </is>
       </c>
       <c r="BU2" t="inlineStr">
         <is>
-          <t>VR6</t>
+          <t>VR11</t>
         </is>
       </c>
       <c r="BV2" t="inlineStr">
         <is>
-          <t>Component / Device</t>
+          <t>Circuit Data</t>
         </is>
       </c>
       <c r="BW2" t="inlineStr">
@@ -1620,7 +1630,7 @@
       </c>
       <c r="BZ2" t="inlineStr">
         <is>
-          <t>Review PhaseConductorId and AveHeightAboveGround_MUL for the section.</t>
+          <t>Review section height/elevation value and confirm whether the value is valid for the conductor type.</t>
         </is>
       </c>
     </row>
@@ -1652,7 +1662,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Conductor height sign does not match the inferred underground or overhead conductor type.</t>
+          <t>Section has negative height or elevation value.</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -1884,17 +1894,17 @@
       </c>
       <c r="BT3" t="inlineStr">
         <is>
-          <t>UG Conductor Height Should Be Negative</t>
+          <t>Section at negative height</t>
         </is>
       </c>
       <c r="BU3" t="inlineStr">
         <is>
-          <t>VR6</t>
+          <t>VR11</t>
         </is>
       </c>
       <c r="BV3" t="inlineStr">
         <is>
-          <t>Component / Device</t>
+          <t>Circuit Data</t>
         </is>
       </c>
       <c r="BW3" t="inlineStr">
@@ -1914,7 +1924,7 @@
       </c>
       <c r="BZ3" t="inlineStr">
         <is>
-          <t>Review PhaseConductorId and AveHeightAboveGround_MUL for the section.</t>
+          <t>Review section height/elevation value and confirm whether the value is valid for the conductor type.</t>
         </is>
       </c>
     </row>
@@ -1946,7 +1956,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Conductor height sign does not match the inferred underground or overhead conductor type.</t>
+          <t>Section has negative height or elevation value.</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -2182,17 +2192,17 @@
       </c>
       <c r="BT4" t="inlineStr">
         <is>
-          <t>UG Conductor Height Should Be Negative</t>
+          <t>Section at negative height</t>
         </is>
       </c>
       <c r="BU4" t="inlineStr">
         <is>
-          <t>VR6</t>
+          <t>VR11</t>
         </is>
       </c>
       <c r="BV4" t="inlineStr">
         <is>
-          <t>Component / Device</t>
+          <t>Circuit Data</t>
         </is>
       </c>
       <c r="BW4" t="inlineStr">
@@ -2212,7 +2222,7 @@
       </c>
       <c r="BZ4" t="inlineStr">
         <is>
-          <t>Review PhaseConductorId and AveHeightAboveGround_MUL for the section.</t>
+          <t>Review section height/elevation value and confirm whether the value is valid for the conductor type.</t>
         </is>
       </c>
     </row>
@@ -2244,7 +2254,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Conductor height sign does not match the inferred underground or overhead conductor type.</t>
+          <t>Section has negative height or elevation value.</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -2476,17 +2486,17 @@
       </c>
       <c r="BT5" t="inlineStr">
         <is>
-          <t>UG Conductor Height Should Be Negative</t>
+          <t>Section at negative height</t>
         </is>
       </c>
       <c r="BU5" t="inlineStr">
         <is>
-          <t>VR6</t>
+          <t>VR11</t>
         </is>
       </c>
       <c r="BV5" t="inlineStr">
         <is>
-          <t>Component / Device</t>
+          <t>Circuit Data</t>
         </is>
       </c>
       <c r="BW5" t="inlineStr">
@@ -2506,7 +2516,7 @@
       </c>
       <c r="BZ5" t="inlineStr">
         <is>
-          <t>Review PhaseConductorId and AveHeightAboveGround_MUL for the section.</t>
+          <t>Review section height/elevation value and confirm whether the value is valid for the conductor type.</t>
         </is>
       </c>
     </row>
@@ -2538,7 +2548,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Conductor height sign does not match the inferred underground or overhead conductor type.</t>
+          <t>Section has negative height or elevation value.</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -2770,17 +2780,17 @@
       </c>
       <c r="BT6" t="inlineStr">
         <is>
-          <t>UG Conductor Height Should Be Negative</t>
+          <t>Section at negative height</t>
         </is>
       </c>
       <c r="BU6" t="inlineStr">
         <is>
-          <t>VR6</t>
+          <t>VR11</t>
         </is>
       </c>
       <c r="BV6" t="inlineStr">
         <is>
-          <t>Component / Device</t>
+          <t>Circuit Data</t>
         </is>
       </c>
       <c r="BW6" t="inlineStr">
@@ -2800,7 +2810,7 @@
       </c>
       <c r="BZ6" t="inlineStr">
         <is>
-          <t>Review PhaseConductorId and AveHeightAboveGround_MUL for the section.</t>
+          <t>Review section height/elevation value and confirm whether the value is valid for the conductor type.</t>
         </is>
       </c>
     </row>
@@ -2832,7 +2842,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Conductor height sign does not match the inferred underground or overhead conductor type.</t>
+          <t>Section has negative height or elevation value.</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -3064,17 +3074,17 @@
       </c>
       <c r="BT7" t="inlineStr">
         <is>
-          <t>UG Conductor Height Should Be Negative</t>
+          <t>Section at negative height</t>
         </is>
       </c>
       <c r="BU7" t="inlineStr">
         <is>
-          <t>VR6</t>
+          <t>VR11</t>
         </is>
       </c>
       <c r="BV7" t="inlineStr">
         <is>
-          <t>Component / Device</t>
+          <t>Circuit Data</t>
         </is>
       </c>
       <c r="BW7" t="inlineStr">
@@ -3094,7 +3104,7 @@
       </c>
       <c r="BZ7" t="inlineStr">
         <is>
-          <t>Review PhaseConductorId and AveHeightAboveGround_MUL for the section.</t>
+          <t>Review section height/elevation value and confirm whether the value is valid for the conductor type.</t>
         </is>
       </c>
     </row>
@@ -3126,7 +3136,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Conductor height sign does not match the inferred underground or overhead conductor type.</t>
+          <t>Section has negative height or elevation value.</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -3350,17 +3360,17 @@
       </c>
       <c r="BT8" t="inlineStr">
         <is>
-          <t>UG Conductor Height Should Be Negative</t>
+          <t>Section at negative height</t>
         </is>
       </c>
       <c r="BU8" t="inlineStr">
         <is>
-          <t>VR6</t>
+          <t>VR11</t>
         </is>
       </c>
       <c r="BV8" t="inlineStr">
         <is>
-          <t>Component / Device</t>
+          <t>Circuit Data</t>
         </is>
       </c>
       <c r="BW8" t="inlineStr">
@@ -3380,7 +3390,7 @@
       </c>
       <c r="BZ8" t="inlineStr">
         <is>
-          <t>Review PhaseConductorId and AveHeightAboveGround_MUL for the section.</t>
+          <t>Review section height/elevation value and confirm whether the value is valid for the conductor type.</t>
         </is>
       </c>
     </row>
@@ -3412,7 +3422,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Conductor height sign does not match the inferred underground or overhead conductor type.</t>
+          <t>Section has negative height or elevation value.</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -3636,17 +3646,17 @@
       </c>
       <c r="BT9" t="inlineStr">
         <is>
-          <t>UG Conductor Height Should Be Negative</t>
+          <t>Section at negative height</t>
         </is>
       </c>
       <c r="BU9" t="inlineStr">
         <is>
-          <t>VR6</t>
+          <t>VR11</t>
         </is>
       </c>
       <c r="BV9" t="inlineStr">
         <is>
-          <t>Component / Device</t>
+          <t>Circuit Data</t>
         </is>
       </c>
       <c r="BW9" t="inlineStr">
@@ -3666,7 +3676,7 @@
       </c>
       <c r="BZ9" t="inlineStr">
         <is>
-          <t>Review PhaseConductorId and AveHeightAboveGround_MUL for the section.</t>
+          <t>Review section height/elevation value and confirm whether the value is valid for the conductor type.</t>
         </is>
       </c>
     </row>
@@ -3698,7 +3708,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Conductor height sign does not match the inferred underground or overhead conductor type.</t>
+          <t>Section has negative height or elevation value.</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -3922,17 +3932,17 @@
       </c>
       <c r="BT10" t="inlineStr">
         <is>
-          <t>UG Conductor Height Should Be Negative</t>
+          <t>Section at negative height</t>
         </is>
       </c>
       <c r="BU10" t="inlineStr">
         <is>
-          <t>VR6</t>
+          <t>VR11</t>
         </is>
       </c>
       <c r="BV10" t="inlineStr">
         <is>
-          <t>Component / Device</t>
+          <t>Circuit Data</t>
         </is>
       </c>
       <c r="BW10" t="inlineStr">
@@ -3952,7 +3962,7 @@
       </c>
       <c r="BZ10" t="inlineStr">
         <is>
-          <t>Review PhaseConductorId and AveHeightAboveGround_MUL for the section.</t>
+          <t>Review section height/elevation value and confirm whether the value is valid for the conductor type.</t>
         </is>
       </c>
     </row>
@@ -4608,11 +4618,7 @@
           <t>CapacitorIssues</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>VR5</t>
-        </is>
-      </c>
+      <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr">
         <is>
           <t>Component / Device</t>
@@ -4635,12 +4641,12 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>&gt;1 MVAR</t>
+          <t>Capacitor greater than 1 MVAR</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Capacitor configuration is outside expected validation limits.</t>
+          <t>Capacitor configured rating is greater than 1 MVAR.</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -4900,11 +4906,7 @@
           <t>CapacitorIssues</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>VR5</t>
-        </is>
-      </c>
+      <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr">
         <is>
           <t>Component / Device</t>
@@ -4927,12 +4929,12 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>&gt;1 MVAR</t>
+          <t>Capacitor greater than 1 MVAR</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Capacitor configuration is outside expected validation limits.</t>
+          <t>Capacitor configured rating is greater than 1 MVAR.</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -5192,11 +5194,7 @@
           <t>CapacitorIssues</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>VR5</t>
-        </is>
-      </c>
+      <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr">
         <is>
           <t>Component / Device</t>
@@ -5219,12 +5217,12 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>&gt;1 MVAR</t>
+          <t>Capacitor greater than 1 MVAR</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Capacitor configuration is outside expected validation limits.</t>
+          <t>Capacitor configured rating is greater than 1 MVAR.</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -5484,11 +5482,7 @@
           <t>CapacitorIssues</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>VR5</t>
-        </is>
-      </c>
+      <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr">
         <is>
           <t>Component / Device</t>
@@ -5511,12 +5505,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>&gt;1 MVAR</t>
+          <t>Capacitor greater than 1 MVAR</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Capacitor configuration is outside expected validation limits.</t>
+          <t>Capacitor configured rating is greater than 1 MVAR.</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -5776,11 +5770,7 @@
           <t>CapacitorIssues</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>VR5</t>
-        </is>
-      </c>
+      <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr">
         <is>
           <t>Component / Device</t>
@@ -5803,12 +5793,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>&gt;1 MVAR</t>
+          <t>Capacitor greater than 1 MVAR</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Capacitor configuration is outside expected validation limits.</t>
+          <t>Capacitor configured rating is greater than 1 MVAR.</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -6068,11 +6058,7 @@
           <t>CapacitorIssues</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>VR5</t>
-        </is>
-      </c>
+      <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr">
         <is>
           <t>Component / Device</t>
@@ -6095,12 +6081,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>&gt;1 MVAR</t>
+          <t>Capacitor greater than 1 MVAR</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Capacitor configuration is outside expected validation limits.</t>
+          <t>Capacitor configured rating is greater than 1 MVAR.</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -6360,11 +6346,7 @@
           <t>CapacitorIssues</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>VR5</t>
-        </is>
-      </c>
+      <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr">
         <is>
           <t>Component / Device</t>
@@ -6387,12 +6369,12 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>&gt;1 MVAR</t>
+          <t>Capacitor greater than 1 MVAR</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Capacitor configuration is outside expected validation limits.</t>
+          <t>Capacitor configured rating is greater than 1 MVAR.</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -6652,11 +6634,7 @@
           <t>CapacitorIssues</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>VR5</t>
-        </is>
-      </c>
+      <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr">
         <is>
           <t>Component / Device</t>
@@ -6679,12 +6657,12 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>&gt;1 MVAR</t>
+          <t>Capacitor greater than 1 MVAR</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Capacitor configuration is outside expected validation limits.</t>
+          <t>Capacitor configured rating is greater than 1 MVAR.</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -6944,11 +6922,7 @@
           <t>CapacitorIssues</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>VR5</t>
-        </is>
-      </c>
+      <c r="B10" t="inlineStr"/>
       <c r="C10" t="inlineStr">
         <is>
           <t>Component / Device</t>
@@ -6971,12 +6945,12 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>&gt;1 MVAR</t>
+          <t>Capacitor greater than 1 MVAR</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>Capacitor configuration is outside expected validation limits.</t>
+          <t>Capacitor configured rating is greater than 1 MVAR.</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -7236,11 +7210,7 @@
           <t>CapacitorIssues</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>VR5</t>
-        </is>
-      </c>
+      <c r="B11" t="inlineStr"/>
       <c r="C11" t="inlineStr">
         <is>
           <t>Component / Device</t>
@@ -7263,12 +7233,12 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>&gt;1 MVAR</t>
+          <t>Capacitor greater than 1 MVAR</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>Capacitor configuration is outside expected validation limits.</t>
+          <t>Capacitor configured rating is greater than 1 MVAR.</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -7530,12 +7500,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>VR6</t>
+          <t>VR11</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Component / Device</t>
+          <t>Circuit Data</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -7555,17 +7525,17 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>UG Conductor Height Should Be Negative</t>
+          <t>Section at negative height</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Conductor height sign does not match the inferred underground or overhead conductor type.</t>
+          <t>Section has negative height or elevation value.</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Review PhaseConductorId and AveHeightAboveGround_MUL for the section.</t>
+          <t>Review section height/elevation value and confirm whether the value is valid for the conductor type.</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
@@ -7876,12 +7846,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>VR6</t>
+          <t>VR11</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Component / Device</t>
+          <t>Circuit Data</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -7901,17 +7871,17 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>UG Conductor Height Should Be Negative</t>
+          <t>Section at negative height</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>Conductor height sign does not match the inferred underground or overhead conductor type.</t>
+          <t>Section has negative height or elevation value.</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>Review PhaseConductorId and AveHeightAboveGround_MUL for the section.</t>
+          <t>Review section height/elevation value and confirm whether the value is valid for the conductor type.</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
@@ -8222,12 +8192,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>VR6</t>
+          <t>VR11</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Component / Device</t>
+          <t>Circuit Data</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -8247,17 +8217,17 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>UG Conductor Height Should Be Negative</t>
+          <t>Section at negative height</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>Conductor height sign does not match the inferred underground or overhead conductor type.</t>
+          <t>Section has negative height or elevation value.</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>Review PhaseConductorId and AveHeightAboveGround_MUL for the section.</t>
+          <t>Review section height/elevation value and confirm whether the value is valid for the conductor type.</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
@@ -8572,12 +8542,12 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>VR6</t>
+          <t>VR11</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Component / Device</t>
+          <t>Circuit Data</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -8597,17 +8567,17 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>UG Conductor Height Should Be Negative</t>
+          <t>Section at negative height</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>Conductor height sign does not match the inferred underground or overhead conductor type.</t>
+          <t>Section has negative height or elevation value.</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>Review PhaseConductorId and AveHeightAboveGround_MUL for the section.</t>
+          <t>Review section height/elevation value and confirm whether the value is valid for the conductor type.</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
@@ -8918,12 +8888,12 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>VR6</t>
+          <t>VR11</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Component / Device</t>
+          <t>Circuit Data</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -8943,17 +8913,17 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>UG Conductor Height Should Be Negative</t>
+          <t>Section at negative height</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>Conductor height sign does not match the inferred underground or overhead conductor type.</t>
+          <t>Section has negative height or elevation value.</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>Review PhaseConductorId and AveHeightAboveGround_MUL for the section.</t>
+          <t>Review section height/elevation value and confirm whether the value is valid for the conductor type.</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
@@ -9264,12 +9234,12 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>VR6</t>
+          <t>VR11</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Component / Device</t>
+          <t>Circuit Data</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -9289,17 +9259,17 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>UG Conductor Height Should Be Negative</t>
+          <t>Section at negative height</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>Conductor height sign does not match the inferred underground or overhead conductor type.</t>
+          <t>Section has negative height or elevation value.</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>Review PhaseConductorId and AveHeightAboveGround_MUL for the section.</t>
+          <t>Review section height/elevation value and confirm whether the value is valid for the conductor type.</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
@@ -9610,12 +9580,12 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>VR6</t>
+          <t>VR11</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Component / Device</t>
+          <t>Circuit Data</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -9635,17 +9605,17 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>UG Conductor Height Should Be Negative</t>
+          <t>Section at negative height</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>Conductor height sign does not match the inferred underground or overhead conductor type.</t>
+          <t>Section has negative height or elevation value.</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>Review PhaseConductorId and AveHeightAboveGround_MUL for the section.</t>
+          <t>Review section height/elevation value and confirm whether the value is valid for the conductor type.</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
@@ -9948,12 +9918,12 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>VR6</t>
+          <t>VR11</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Component / Device</t>
+          <t>Circuit Data</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -9973,17 +9943,17 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>UG Conductor Height Should Be Negative</t>
+          <t>Section at negative height</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>Conductor height sign does not match the inferred underground or overhead conductor type.</t>
+          <t>Section has negative height or elevation value.</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>Review PhaseConductorId and AveHeightAboveGround_MUL for the section.</t>
+          <t>Review section height/elevation value and confirm whether the value is valid for the conductor type.</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
@@ -10286,12 +10256,12 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>VR6</t>
+          <t>VR11</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Component / Device</t>
+          <t>Circuit Data</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -10311,17 +10281,17 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>UG Conductor Height Should Be Negative</t>
+          <t>Section at negative height</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>Conductor height sign does not match the inferred underground or overhead conductor type.</t>
+          <t>Section has negative height or elevation value.</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>Review PhaseConductorId and AveHeightAboveGround_MUL for the section.</t>
+          <t>Review section height/elevation value and confirm whether the value is valid for the conductor type.</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
@@ -12663,385 +12633,397 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>RuleID</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Severity</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>ElementType</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>ElementID</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Issue</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>RecommendedAction</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
           <t>SectionId</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>UniqueDeviceId</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>ConnectedPhases</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>ConnectionType</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>MeteringPhase</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>PrimaryControlMode</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>CapacitorIsOn</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>ManualOperation</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>FixedKvarPhase1</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>FixedKvarPhase2</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>FixedKvarPhase3</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>Module1On</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>Module1Activated</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>Module1KvarPerPhase</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>Module1CapSwitchCloseValue</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>Module1CapSwitchTripValue</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>Module2On</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>Module2Activated</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>Module2KvarPerPhase</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="AB1" t="inlineStr">
         <is>
           <t>Module2CapSwitchCloseValue</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="AC1" t="inlineStr">
         <is>
           <t>Module2CapSwitchTripValue</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="AD1" t="inlineStr">
         <is>
           <t>Module3On</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="AE1" t="inlineStr">
         <is>
           <t>Module3Activated</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="AF1" t="inlineStr">
         <is>
           <t>Module3KvarPerPhase</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="AG1" t="inlineStr">
         <is>
           <t>Module3CapSwitchCloseValue</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="AH1" t="inlineStr">
         <is>
           <t>Module3CapSwitchTripValue</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AI1" t="inlineStr">
         <is>
           <t>CapacitorRDial</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AJ1" t="inlineStr">
         <is>
           <t>CapacitorXDial</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AK1" t="inlineStr">
         <is>
           <t>CapacitorPTRatio</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AL1" t="inlineStr">
         <is>
           <t>CapacitorCTRating</t>
         </is>
       </c>
-      <c r="AE1" t="inlineStr">
+      <c r="AM1" t="inlineStr">
         <is>
           <t>CapVoltageOverrideActive</t>
         </is>
       </c>
-      <c r="AF1" t="inlineStr">
+      <c r="AN1" t="inlineStr">
         <is>
           <t>CapVoltageOverrideSetting</t>
         </is>
       </c>
-      <c r="AG1" t="inlineStr">
+      <c r="AO1" t="inlineStr">
         <is>
           <t>CapVoltageOverrideBandwidth</t>
         </is>
       </c>
-      <c r="AH1" t="inlineStr">
+      <c r="AP1" t="inlineStr">
         <is>
           <t>LocationLink</t>
         </is>
       </c>
-      <c r="AI1" t="inlineStr">
+      <c r="AQ1" t="inlineStr">
         <is>
           <t>TimeCtrlOffOnWeekEnds</t>
         </is>
       </c>
-      <c r="AJ1" t="inlineStr">
+      <c r="AR1" t="inlineStr">
         <is>
           <t>RatedKv</t>
         </is>
       </c>
-      <c r="AK1" t="inlineStr">
+      <c r="AS1" t="inlineStr">
         <is>
           <t>EnergizeYear</t>
         </is>
       </c>
-      <c r="AL1" t="inlineStr">
+      <c r="AT1" t="inlineStr">
         <is>
           <t>RetireYear</t>
         </is>
       </c>
-      <c r="AM1" t="inlineStr">
+      <c r="AU1" t="inlineStr">
         <is>
           <t>Note_</t>
         </is>
       </c>
-      <c r="AN1" t="inlineStr">
+      <c r="AV1" t="inlineStr">
         <is>
           <t>AMSLink</t>
         </is>
       </c>
-      <c r="AO1" t="inlineStr">
+      <c r="AW1" t="inlineStr">
         <is>
           <t>SubOperSeq</t>
         </is>
       </c>
-      <c r="AP1" t="inlineStr">
+      <c r="AX1" t="inlineStr">
         <is>
           <t>TimeDelaySec</t>
         </is>
       </c>
-      <c r="AQ1" t="inlineStr">
+      <c r="AY1" t="inlineStr">
         <is>
           <t>StatcomIsActive</t>
         </is>
       </c>
-      <c r="AR1" t="inlineStr">
+      <c r="AZ1" t="inlineStr">
         <is>
           <t>StatcomVoltSet</t>
         </is>
       </c>
-      <c r="AS1" t="inlineStr">
+      <c r="BA1" t="inlineStr">
         <is>
           <t>StatcomKvarPrVolt</t>
         </is>
       </c>
-      <c r="AT1" t="inlineStr">
+      <c r="BB1" t="inlineStr">
         <is>
           <t>StatcomMaxCap</t>
         </is>
       </c>
-      <c r="AU1" t="inlineStr">
+      <c r="BC1" t="inlineStr">
         <is>
           <t>StatcomMaxInd</t>
         </is>
       </c>
-      <c r="AV1" t="inlineStr">
+      <c r="BD1" t="inlineStr">
         <is>
           <t>WhatIfCode</t>
         </is>
       </c>
-      <c r="AW1" t="inlineStr">
+      <c r="BE1" t="inlineStr">
         <is>
           <t>Module1NormOn</t>
         </is>
       </c>
-      <c r="AX1" t="inlineStr">
+      <c r="BF1" t="inlineStr">
         <is>
           <t>Module2NormOn</t>
         </is>
       </c>
-      <c r="AY1" t="inlineStr">
+      <c r="BG1" t="inlineStr">
         <is>
           <t>Module3NormOn</t>
         </is>
       </c>
-      <c r="AZ1" t="inlineStr">
+      <c r="BH1" t="inlineStr">
         <is>
           <t>TotalFixedKvar</t>
         </is>
       </c>
-      <c r="BA1" t="inlineStr">
+      <c r="BI1" t="inlineStr">
         <is>
           <t>TotalSwitchedKvar</t>
         </is>
       </c>
-      <c r="BB1" t="inlineStr">
+      <c r="BJ1" t="inlineStr">
         <is>
           <t>TotalKvar</t>
-        </is>
-      </c>
-      <c r="BC1" t="inlineStr">
-        <is>
-          <t>Issue</t>
-        </is>
-      </c>
-      <c r="BD1" t="inlineStr">
-        <is>
-          <t>RuleID</t>
-        </is>
-      </c>
-      <c r="BE1" t="inlineStr">
-        <is>
-          <t>Category</t>
-        </is>
-      </c>
-      <c r="BF1" t="inlineStr">
-        <is>
-          <t>Severity</t>
-        </is>
-      </c>
-      <c r="BG1" t="inlineStr">
-        <is>
-          <t>ElementType</t>
-        </is>
-      </c>
-      <c r="BH1" t="inlineStr">
-        <is>
-          <t>ElementID</t>
-        </is>
-      </c>
-      <c r="BI1" t="inlineStr">
-        <is>
-          <t>Description</t>
-        </is>
-      </c>
-      <c r="BJ1" t="inlineStr">
-        <is>
-          <t>RecommendedAction</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" t="inlineStr"/>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Component / Device</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Warning</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Capacitor</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Cap Dkn_001</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Capacitor greater than 1 MVAR</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Capacitor configured rating is greater than 1 MVAR.</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Review capacitor KVAR settings and confirm the converted model values.</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
         <is>
           <t>Dkn_00053</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>Cap Dkn_001</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>ABC</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="L2" t="inlineStr">
         <is>
           <t>YG</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="M2" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="N2" t="inlineStr">
         <is>
           <t>PF</t>
         </is>
       </c>
-      <c r="G2" t="n">
-        <v>1</v>
-      </c>
-      <c r="H2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I2" t="n">
+      <c r="O2" t="n">
+        <v>1</v>
+      </c>
+      <c r="P2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q2" t="n">
         <v>400</v>
       </c>
-      <c r="J2" t="n">
+      <c r="R2" t="n">
         <v>400</v>
       </c>
-      <c r="K2" t="n">
+      <c r="S2" t="n">
         <v>400</v>
       </c>
-      <c r="L2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R2" t="n">
-        <v>0</v>
-      </c>
-      <c r="S2" t="n">
-        <v>0</v>
-      </c>
       <c r="T2" t="n">
         <v>0</v>
       </c>
@@ -13084,188 +13066,184 @@
       <c r="AG2" t="n">
         <v>0</v>
       </c>
-      <c r="AH2" t="inlineStr">
+      <c r="AH2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP2" t="inlineStr">
         <is>
           <t>*</t>
         </is>
       </c>
-      <c r="AI2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AK2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AL2" t="n">
+      <c r="AQ2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT2" t="n">
         <v>100</v>
       </c>
-      <c r="AM2" t="inlineStr">
+      <c r="AU2" t="inlineStr">
         <is>
           <t> </t>
         </is>
       </c>
-      <c r="AN2" t="inlineStr">
+      <c r="AV2" t="inlineStr">
         <is>
           <t> </t>
         </is>
       </c>
-      <c r="AO2" t="n">
-        <v>1</v>
-      </c>
-      <c r="AP2" t="n">
+      <c r="AW2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX2" t="n">
         <v>300</v>
       </c>
-      <c r="AQ2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AR2" t="n">
+      <c r="AY2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ2" t="n">
         <v>122</v>
       </c>
-      <c r="AS2" t="n">
+      <c r="BA2" t="n">
         <v>600</v>
-      </c>
-      <c r="AT2" t="n">
-        <v>1200</v>
-      </c>
-      <c r="AU2" t="n">
-        <v>1200</v>
-      </c>
-      <c r="AV2" t="inlineStr">
-        <is>
-          <t> </t>
-        </is>
-      </c>
-      <c r="AW2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AX2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AY2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AZ2" t="n">
-        <v>1200</v>
-      </c>
-      <c r="BA2" t="n">
-        <v>0</v>
       </c>
       <c r="BB2" t="n">
         <v>1200</v>
       </c>
-      <c r="BC2" t="inlineStr">
-        <is>
-          <t>&gt;1 MVAR</t>
-        </is>
+      <c r="BC2" t="n">
+        <v>1200</v>
       </c>
       <c r="BD2" t="inlineStr">
         <is>
-          <t>VR5</t>
-        </is>
-      </c>
-      <c r="BE2" t="inlineStr">
-        <is>
-          <t>Component / Device</t>
-        </is>
-      </c>
-      <c r="BF2" t="inlineStr">
-        <is>
-          <t>Warning</t>
-        </is>
-      </c>
-      <c r="BG2" t="inlineStr">
-        <is>
-          <t>Capacitor</t>
-        </is>
-      </c>
-      <c r="BH2" t="inlineStr">
-        <is>
-          <t>Cap Dkn_001</t>
-        </is>
-      </c>
-      <c r="BI2" t="inlineStr">
-        <is>
-          <t>Capacitor configuration is outside expected validation limits.</t>
-        </is>
-      </c>
-      <c r="BJ2" t="inlineStr">
-        <is>
-          <t>Review capacitor KVAR settings and confirm the converted model values.</t>
-        </is>
+          <t> </t>
+        </is>
+      </c>
+      <c r="BE2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH2" t="n">
+        <v>1200</v>
+      </c>
+      <c r="BI2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ2" t="n">
+        <v>1200</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" t="inlineStr"/>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Component / Device</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Warning</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Capacitor</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Cap Dkn_003</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Capacitor greater than 1 MVAR</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Capacitor configured rating is greater than 1 MVAR.</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Review capacitor KVAR settings and confirm the converted model values.</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
         <is>
           <t>Dkn_00151</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="J3" t="inlineStr">
         <is>
           <t>Cap Dkn_003</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="K3" t="inlineStr">
         <is>
           <t>ABC</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="L3" t="inlineStr">
         <is>
           <t>YG</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="M3" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="N3" t="inlineStr">
         <is>
           <t>PF</t>
         </is>
       </c>
-      <c r="G3" t="n">
-        <v>1</v>
-      </c>
-      <c r="H3" t="n">
-        <v>0</v>
-      </c>
-      <c r="I3" t="n">
+      <c r="O3" t="n">
+        <v>1</v>
+      </c>
+      <c r="P3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q3" t="n">
         <v>600</v>
       </c>
-      <c r="J3" t="n">
+      <c r="R3" t="n">
         <v>600</v>
       </c>
-      <c r="K3" t="n">
+      <c r="S3" t="n">
         <v>600</v>
       </c>
-      <c r="L3" t="n">
-        <v>0</v>
-      </c>
-      <c r="M3" t="n">
-        <v>0</v>
-      </c>
-      <c r="N3" t="n">
-        <v>0</v>
-      </c>
-      <c r="O3" t="n">
-        <v>0</v>
-      </c>
-      <c r="P3" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q3" t="n">
-        <v>0</v>
-      </c>
-      <c r="R3" t="n">
-        <v>0</v>
-      </c>
-      <c r="S3" t="n">
-        <v>0</v>
-      </c>
       <c r="T3" t="n">
         <v>0</v>
       </c>
@@ -13308,188 +13286,184 @@
       <c r="AG3" t="n">
         <v>0</v>
       </c>
-      <c r="AH3" t="inlineStr">
+      <c r="AH3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP3" t="inlineStr">
         <is>
           <t>*</t>
         </is>
       </c>
-      <c r="AI3" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ3" t="n">
-        <v>0</v>
-      </c>
-      <c r="AK3" t="n">
-        <v>0</v>
-      </c>
-      <c r="AL3" t="n">
+      <c r="AQ3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT3" t="n">
         <v>100</v>
       </c>
-      <c r="AM3" t="inlineStr">
+      <c r="AU3" t="inlineStr">
         <is>
           <t> </t>
         </is>
       </c>
-      <c r="AN3" t="inlineStr">
+      <c r="AV3" t="inlineStr">
         <is>
           <t> </t>
         </is>
       </c>
-      <c r="AO3" t="n">
-        <v>1</v>
-      </c>
-      <c r="AP3" t="n">
+      <c r="AW3" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX3" t="n">
         <v>300</v>
       </c>
-      <c r="AQ3" t="n">
-        <v>0</v>
-      </c>
-      <c r="AR3" t="n">
+      <c r="AY3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ3" t="n">
         <v>122</v>
       </c>
-      <c r="AS3" t="n">
+      <c r="BA3" t="n">
         <v>600</v>
       </c>
-      <c r="AT3" t="n">
+      <c r="BB3" t="n">
         <v>1200</v>
       </c>
-      <c r="AU3" t="n">
+      <c r="BC3" t="n">
         <v>1200</v>
       </c>
-      <c r="AV3" t="inlineStr">
+      <c r="BD3" t="inlineStr">
         <is>
           <t> </t>
         </is>
       </c>
-      <c r="AW3" t="n">
-        <v>0</v>
-      </c>
-      <c r="AX3" t="n">
-        <v>0</v>
-      </c>
-      <c r="AY3" t="n">
-        <v>0</v>
-      </c>
-      <c r="AZ3" t="n">
+      <c r="BE3" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF3" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG3" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH3" t="n">
         <v>1800</v>
       </c>
-      <c r="BA3" t="n">
-        <v>0</v>
-      </c>
-      <c r="BB3" t="n">
+      <c r="BI3" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ3" t="n">
         <v>1800</v>
-      </c>
-      <c r="BC3" t="inlineStr">
-        <is>
-          <t>&gt;1 MVAR</t>
-        </is>
-      </c>
-      <c r="BD3" t="inlineStr">
-        <is>
-          <t>VR5</t>
-        </is>
-      </c>
-      <c r="BE3" t="inlineStr">
-        <is>
-          <t>Component / Device</t>
-        </is>
-      </c>
-      <c r="BF3" t="inlineStr">
-        <is>
-          <t>Warning</t>
-        </is>
-      </c>
-      <c r="BG3" t="inlineStr">
-        <is>
-          <t>Capacitor</t>
-        </is>
-      </c>
-      <c r="BH3" t="inlineStr">
-        <is>
-          <t>Cap Dkn_003</t>
-        </is>
-      </c>
-      <c r="BI3" t="inlineStr">
-        <is>
-          <t>Capacitor configuration is outside expected validation limits.</t>
-        </is>
-      </c>
-      <c r="BJ3" t="inlineStr">
-        <is>
-          <t>Review capacitor KVAR settings and confirm the converted model values.</t>
-        </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" t="inlineStr"/>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Component / Device</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Warning</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Capacitor</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Cap Dkn_004</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Capacitor greater than 1 MVAR</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Capacitor configured rating is greater than 1 MVAR.</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Review capacitor KVAR settings and confirm the converted model values.</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
         <is>
           <t>Dkn_00153</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="J4" t="inlineStr">
         <is>
           <t>Cap Dkn_004</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="K4" t="inlineStr">
         <is>
           <t>ABC</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="L4" t="inlineStr">
         <is>
           <t>YG</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="M4" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="N4" t="inlineStr">
         <is>
           <t>PF</t>
         </is>
       </c>
-      <c r="G4" t="n">
-        <v>1</v>
-      </c>
-      <c r="H4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I4" t="n">
+      <c r="O4" t="n">
+        <v>1</v>
+      </c>
+      <c r="P4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q4" t="n">
         <v>400</v>
       </c>
-      <c r="J4" t="n">
+      <c r="R4" t="n">
         <v>400</v>
       </c>
-      <c r="K4" t="n">
+      <c r="S4" t="n">
         <v>400</v>
       </c>
-      <c r="L4" t="n">
-        <v>0</v>
-      </c>
-      <c r="M4" t="n">
-        <v>0</v>
-      </c>
-      <c r="N4" t="n">
-        <v>0</v>
-      </c>
-      <c r="O4" t="n">
-        <v>0</v>
-      </c>
-      <c r="P4" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q4" t="n">
-        <v>0</v>
-      </c>
-      <c r="R4" t="n">
-        <v>0</v>
-      </c>
-      <c r="S4" t="n">
-        <v>0</v>
-      </c>
       <c r="T4" t="n">
         <v>0</v>
       </c>
@@ -13532,188 +13506,184 @@
       <c r="AG4" t="n">
         <v>0</v>
       </c>
-      <c r="AH4" t="inlineStr">
+      <c r="AH4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP4" t="inlineStr">
         <is>
           <t>*</t>
         </is>
       </c>
-      <c r="AI4" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ4" t="n">
-        <v>0</v>
-      </c>
-      <c r="AK4" t="n">
-        <v>0</v>
-      </c>
-      <c r="AL4" t="n">
+      <c r="AQ4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT4" t="n">
         <v>100</v>
       </c>
-      <c r="AM4" t="inlineStr">
+      <c r="AU4" t="inlineStr">
         <is>
           <t> </t>
         </is>
       </c>
-      <c r="AN4" t="inlineStr">
+      <c r="AV4" t="inlineStr">
         <is>
           <t> </t>
         </is>
       </c>
-      <c r="AO4" t="n">
-        <v>1</v>
-      </c>
-      <c r="AP4" t="n">
+      <c r="AW4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX4" t="n">
         <v>300</v>
       </c>
-      <c r="AQ4" t="n">
-        <v>0</v>
-      </c>
-      <c r="AR4" t="n">
+      <c r="AY4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ4" t="n">
         <v>122</v>
       </c>
-      <c r="AS4" t="n">
+      <c r="BA4" t="n">
         <v>600</v>
-      </c>
-      <c r="AT4" t="n">
-        <v>1200</v>
-      </c>
-      <c r="AU4" t="n">
-        <v>1200</v>
-      </c>
-      <c r="AV4" t="inlineStr">
-        <is>
-          <t> </t>
-        </is>
-      </c>
-      <c r="AW4" t="n">
-        <v>0</v>
-      </c>
-      <c r="AX4" t="n">
-        <v>0</v>
-      </c>
-      <c r="AY4" t="n">
-        <v>0</v>
-      </c>
-      <c r="AZ4" t="n">
-        <v>1200</v>
-      </c>
-      <c r="BA4" t="n">
-        <v>0</v>
       </c>
       <c r="BB4" t="n">
         <v>1200</v>
       </c>
-      <c r="BC4" t="inlineStr">
-        <is>
-          <t>&gt;1 MVAR</t>
-        </is>
+      <c r="BC4" t="n">
+        <v>1200</v>
       </c>
       <c r="BD4" t="inlineStr">
         <is>
-          <t>VR5</t>
-        </is>
-      </c>
-      <c r="BE4" t="inlineStr">
-        <is>
-          <t>Component / Device</t>
-        </is>
-      </c>
-      <c r="BF4" t="inlineStr">
-        <is>
-          <t>Warning</t>
-        </is>
-      </c>
-      <c r="BG4" t="inlineStr">
-        <is>
-          <t>Capacitor</t>
-        </is>
-      </c>
-      <c r="BH4" t="inlineStr">
-        <is>
-          <t>Cap Dkn_004</t>
-        </is>
-      </c>
-      <c r="BI4" t="inlineStr">
-        <is>
-          <t>Capacitor configuration is outside expected validation limits.</t>
-        </is>
-      </c>
-      <c r="BJ4" t="inlineStr">
-        <is>
-          <t>Review capacitor KVAR settings and confirm the converted model values.</t>
-        </is>
+          <t> </t>
+        </is>
+      </c>
+      <c r="BE4" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF4" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG4" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH4" t="n">
+        <v>1200</v>
+      </c>
+      <c r="BI4" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ4" t="n">
+        <v>1200</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" t="inlineStr"/>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Component / Device</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Warning</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Capacitor</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Cap Dkn_002</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Capacitor greater than 1 MVAR</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Capacitor configured rating is greater than 1 MVAR.</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Review capacitor KVAR settings and confirm the converted model values.</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
         <is>
           <t>Dkn_00172</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="J5" t="inlineStr">
         <is>
           <t>Cap Dkn_002</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="K5" t="inlineStr">
         <is>
           <t>ABC</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="L5" t="inlineStr">
         <is>
           <t>YG</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="M5" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="N5" t="inlineStr">
         <is>
           <t>PF</t>
         </is>
       </c>
-      <c r="G5" t="n">
-        <v>1</v>
-      </c>
-      <c r="H5" t="n">
-        <v>0</v>
-      </c>
-      <c r="I5" t="n">
+      <c r="O5" t="n">
+        <v>1</v>
+      </c>
+      <c r="P5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q5" t="n">
         <v>400</v>
       </c>
-      <c r="J5" t="n">
+      <c r="R5" t="n">
         <v>400</v>
       </c>
-      <c r="K5" t="n">
+      <c r="S5" t="n">
         <v>400</v>
       </c>
-      <c r="L5" t="n">
-        <v>0</v>
-      </c>
-      <c r="M5" t="n">
-        <v>0</v>
-      </c>
-      <c r="N5" t="n">
-        <v>0</v>
-      </c>
-      <c r="O5" t="n">
-        <v>0</v>
-      </c>
-      <c r="P5" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q5" t="n">
-        <v>0</v>
-      </c>
-      <c r="R5" t="n">
-        <v>0</v>
-      </c>
-      <c r="S5" t="n">
-        <v>0</v>
-      </c>
       <c r="T5" t="n">
         <v>0</v>
       </c>
@@ -13756,188 +13726,184 @@
       <c r="AG5" t="n">
         <v>0</v>
       </c>
-      <c r="AH5" t="inlineStr">
+      <c r="AH5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP5" t="inlineStr">
         <is>
           <t>*</t>
         </is>
       </c>
-      <c r="AI5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AK5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AL5" t="n">
+      <c r="AQ5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT5" t="n">
         <v>100</v>
       </c>
-      <c r="AM5" t="inlineStr">
+      <c r="AU5" t="inlineStr">
         <is>
           <t> </t>
         </is>
       </c>
-      <c r="AN5" t="inlineStr">
+      <c r="AV5" t="inlineStr">
         <is>
           <t> </t>
         </is>
       </c>
-      <c r="AO5" t="n">
-        <v>1</v>
-      </c>
-      <c r="AP5" t="n">
+      <c r="AW5" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX5" t="n">
         <v>300</v>
       </c>
-      <c r="AQ5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AR5" t="n">
+      <c r="AY5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ5" t="n">
         <v>122</v>
       </c>
-      <c r="AS5" t="n">
+      <c r="BA5" t="n">
         <v>600</v>
-      </c>
-      <c r="AT5" t="n">
-        <v>1200</v>
-      </c>
-      <c r="AU5" t="n">
-        <v>1200</v>
-      </c>
-      <c r="AV5" t="inlineStr">
-        <is>
-          <t> </t>
-        </is>
-      </c>
-      <c r="AW5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AX5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AY5" t="n">
-        <v>0</v>
-      </c>
-      <c r="AZ5" t="n">
-        <v>1200</v>
-      </c>
-      <c r="BA5" t="n">
-        <v>0</v>
       </c>
       <c r="BB5" t="n">
         <v>1200</v>
       </c>
-      <c r="BC5" t="inlineStr">
-        <is>
-          <t>&gt;1 MVAR</t>
-        </is>
+      <c r="BC5" t="n">
+        <v>1200</v>
       </c>
       <c r="BD5" t="inlineStr">
         <is>
-          <t>VR5</t>
-        </is>
-      </c>
-      <c r="BE5" t="inlineStr">
-        <is>
-          <t>Component / Device</t>
-        </is>
-      </c>
-      <c r="BF5" t="inlineStr">
-        <is>
-          <t>Warning</t>
-        </is>
-      </c>
-      <c r="BG5" t="inlineStr">
-        <is>
-          <t>Capacitor</t>
-        </is>
-      </c>
-      <c r="BH5" t="inlineStr">
-        <is>
-          <t>Cap Dkn_002</t>
-        </is>
-      </c>
-      <c r="BI5" t="inlineStr">
-        <is>
-          <t>Capacitor configuration is outside expected validation limits.</t>
-        </is>
-      </c>
-      <c r="BJ5" t="inlineStr">
-        <is>
-          <t>Review capacitor KVAR settings and confirm the converted model values.</t>
-        </is>
+          <t> </t>
+        </is>
+      </c>
+      <c r="BE5" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF5" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG5" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH5" t="n">
+        <v>1200</v>
+      </c>
+      <c r="BI5" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ5" t="n">
+        <v>1200</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" t="inlineStr"/>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Component / Device</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Warning</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Capacitor</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Cap Dkn_005</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Capacitor greater than 1 MVAR</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Capacitor configured rating is greater than 1 MVAR.</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Review capacitor KVAR settings and confirm the converted model values.</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
         <is>
           <t>Dkn_00217</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="J6" t="inlineStr">
         <is>
           <t>Cap Dkn_005</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="K6" t="inlineStr">
         <is>
           <t>ABC</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="L6" t="inlineStr">
         <is>
           <t>YG</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="M6" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="N6" t="inlineStr">
         <is>
           <t>PF</t>
         </is>
       </c>
-      <c r="G6" t="n">
-        <v>1</v>
-      </c>
-      <c r="H6" t="n">
-        <v>0</v>
-      </c>
-      <c r="I6" t="n">
+      <c r="O6" t="n">
+        <v>1</v>
+      </c>
+      <c r="P6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q6" t="n">
         <v>600</v>
       </c>
-      <c r="J6" t="n">
+      <c r="R6" t="n">
         <v>600</v>
       </c>
-      <c r="K6" t="n">
+      <c r="S6" t="n">
         <v>600</v>
       </c>
-      <c r="L6" t="n">
-        <v>0</v>
-      </c>
-      <c r="M6" t="n">
-        <v>0</v>
-      </c>
-      <c r="N6" t="n">
-        <v>0</v>
-      </c>
-      <c r="O6" t="n">
-        <v>0</v>
-      </c>
-      <c r="P6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q6" t="n">
-        <v>0</v>
-      </c>
-      <c r="R6" t="n">
-        <v>0</v>
-      </c>
-      <c r="S6" t="n">
-        <v>0</v>
-      </c>
       <c r="T6" t="n">
         <v>0</v>
       </c>
@@ -13980,203 +13946,199 @@
       <c r="AG6" t="n">
         <v>0</v>
       </c>
-      <c r="AH6" t="inlineStr">
+      <c r="AH6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP6" t="inlineStr">
         <is>
           <t>*</t>
         </is>
       </c>
-      <c r="AI6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AK6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AL6" t="n">
+      <c r="AQ6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT6" t="n">
         <v>100</v>
       </c>
-      <c r="AM6" t="inlineStr">
+      <c r="AU6" t="inlineStr">
         <is>
           <t> </t>
         </is>
       </c>
-      <c r="AN6" t="inlineStr">
+      <c r="AV6" t="inlineStr">
         <is>
           <t> </t>
         </is>
       </c>
-      <c r="AO6" t="n">
-        <v>1</v>
-      </c>
-      <c r="AP6" t="n">
+      <c r="AW6" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX6" t="n">
         <v>300</v>
       </c>
-      <c r="AQ6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AR6" t="n">
+      <c r="AY6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ6" t="n">
         <v>122</v>
       </c>
-      <c r="AS6" t="n">
+      <c r="BA6" t="n">
         <v>600</v>
       </c>
-      <c r="AT6" t="n">
+      <c r="BB6" t="n">
         <v>1200</v>
       </c>
-      <c r="AU6" t="n">
+      <c r="BC6" t="n">
         <v>1200</v>
       </c>
-      <c r="AV6" t="inlineStr">
+      <c r="BD6" t="inlineStr">
         <is>
           <t> </t>
         </is>
       </c>
-      <c r="AW6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AX6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AY6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AZ6" t="n">
+      <c r="BE6" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF6" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG6" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH6" t="n">
         <v>1800</v>
       </c>
-      <c r="BA6" t="n">
-        <v>0</v>
-      </c>
-      <c r="BB6" t="n">
+      <c r="BI6" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ6" t="n">
         <v>1800</v>
-      </c>
-      <c r="BC6" t="inlineStr">
-        <is>
-          <t>&gt;1 MVAR</t>
-        </is>
-      </c>
-      <c r="BD6" t="inlineStr">
-        <is>
-          <t>VR5</t>
-        </is>
-      </c>
-      <c r="BE6" t="inlineStr">
-        <is>
-          <t>Component / Device</t>
-        </is>
-      </c>
-      <c r="BF6" t="inlineStr">
-        <is>
-          <t>Warning</t>
-        </is>
-      </c>
-      <c r="BG6" t="inlineStr">
-        <is>
-          <t>Capacitor</t>
-        </is>
-      </c>
-      <c r="BH6" t="inlineStr">
-        <is>
-          <t>Cap Dkn_005</t>
-        </is>
-      </c>
-      <c r="BI6" t="inlineStr">
-        <is>
-          <t>Capacitor configuration is outside expected validation limits.</t>
-        </is>
-      </c>
-      <c r="BJ6" t="inlineStr">
-        <is>
-          <t>Review capacitor KVAR settings and confirm the converted model values.</t>
-        </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" t="inlineStr"/>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Component / Device</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Warning</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Capacitor</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Cap Dkn_006</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Capacitor greater than 1 MVAR</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Capacitor configured rating is greater than 1 MVAR.</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Review capacitor KVAR settings and confirm the converted model values.</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
         <is>
           <t>Dkn_00276</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="J7" t="inlineStr">
         <is>
           <t>Cap Dkn_006</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="K7" t="inlineStr">
         <is>
           <t>ABC</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="L7" t="inlineStr">
         <is>
           <t>YG</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="M7" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="N7" t="inlineStr">
         <is>
           <t>VOLTS</t>
         </is>
       </c>
-      <c r="G7" t="n">
-        <v>1</v>
-      </c>
-      <c r="H7" t="n">
-        <v>0</v>
-      </c>
-      <c r="I7" t="n">
+      <c r="O7" t="n">
+        <v>1</v>
+      </c>
+      <c r="P7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q7" t="n">
         <v>600</v>
       </c>
-      <c r="J7" t="n">
+      <c r="R7" t="n">
         <v>600</v>
       </c>
-      <c r="K7" t="n">
+      <c r="S7" t="n">
         <v>600</v>
       </c>
-      <c r="L7" t="n">
-        <v>0</v>
-      </c>
-      <c r="M7" t="n">
-        <v>1</v>
-      </c>
-      <c r="N7" t="n">
+      <c r="T7" t="n">
+        <v>0</v>
+      </c>
+      <c r="U7" t="n">
+        <v>1</v>
+      </c>
+      <c r="V7" t="n">
         <v>400</v>
       </c>
-      <c r="O7" t="n">
+      <c r="W7" t="n">
         <v>118</v>
       </c>
-      <c r="P7" t="n">
+      <c r="X7" t="n">
         <v>120</v>
       </c>
-      <c r="Q7" t="n">
-        <v>0</v>
-      </c>
-      <c r="R7" t="n">
-        <v>0</v>
-      </c>
-      <c r="S7" t="n">
-        <v>0</v>
-      </c>
-      <c r="T7" t="n">
-        <v>0</v>
-      </c>
-      <c r="U7" t="n">
-        <v>0</v>
-      </c>
-      <c r="V7" t="n">
-        <v>0</v>
-      </c>
-      <c r="W7" t="n">
-        <v>0</v>
-      </c>
-      <c r="X7" t="n">
-        <v>0</v>
-      </c>
       <c r="Y7" t="n">
         <v>0</v>
       </c>
@@ -14190,217 +14152,213 @@
         <v>0</v>
       </c>
       <c r="AC7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK7" t="n">
         <v>165.833</v>
       </c>
-      <c r="AD7" t="n">
+      <c r="AL7" t="n">
         <v>120</v>
       </c>
-      <c r="AE7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH7" t="inlineStr">
+      <c r="AM7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP7" t="inlineStr">
         <is>
           <t>*</t>
         </is>
       </c>
-      <c r="AI7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AK7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AL7" t="n">
+      <c r="AQ7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT7" t="n">
         <v>100</v>
       </c>
-      <c r="AM7" t="inlineStr">
+      <c r="AU7" t="inlineStr">
         <is>
           <t> </t>
         </is>
       </c>
-      <c r="AN7" t="inlineStr">
+      <c r="AV7" t="inlineStr">
         <is>
           <t> </t>
         </is>
       </c>
-      <c r="AO7" t="n">
-        <v>1</v>
-      </c>
-      <c r="AP7" t="n">
+      <c r="AW7" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX7" t="n">
         <v>300</v>
       </c>
-      <c r="AQ7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AR7" t="n">
+      <c r="AY7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ7" t="n">
         <v>122</v>
       </c>
-      <c r="AS7" t="n">
+      <c r="BA7" t="n">
         <v>600</v>
       </c>
-      <c r="AT7" t="n">
+      <c r="BB7" t="n">
         <v>1200</v>
       </c>
-      <c r="AU7" t="n">
+      <c r="BC7" t="n">
         <v>1200</v>
       </c>
-      <c r="AV7" t="inlineStr">
+      <c r="BD7" t="inlineStr">
         <is>
           <t> </t>
         </is>
       </c>
-      <c r="AW7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AX7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AY7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AZ7" t="n">
+      <c r="BE7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH7" t="n">
         <v>1800</v>
       </c>
-      <c r="BA7" t="n">
+      <c r="BI7" t="n">
         <v>400</v>
       </c>
-      <c r="BB7" t="n">
+      <c r="BJ7" t="n">
         <v>2200</v>
-      </c>
-      <c r="BC7" t="inlineStr">
-        <is>
-          <t>&gt;1 MVAR</t>
-        </is>
-      </c>
-      <c r="BD7" t="inlineStr">
-        <is>
-          <t>VR5</t>
-        </is>
-      </c>
-      <c r="BE7" t="inlineStr">
-        <is>
-          <t>Component / Device</t>
-        </is>
-      </c>
-      <c r="BF7" t="inlineStr">
-        <is>
-          <t>Warning</t>
-        </is>
-      </c>
-      <c r="BG7" t="inlineStr">
-        <is>
-          <t>Capacitor</t>
-        </is>
-      </c>
-      <c r="BH7" t="inlineStr">
-        <is>
-          <t>Cap Dkn_006</t>
-        </is>
-      </c>
-      <c r="BI7" t="inlineStr">
-        <is>
-          <t>Capacitor configuration is outside expected validation limits.</t>
-        </is>
-      </c>
-      <c r="BJ7" t="inlineStr">
-        <is>
-          <t>Review capacitor KVAR settings and confirm the converted model values.</t>
-        </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" t="inlineStr"/>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Component / Device</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Warning</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Capacitor</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Cap Dkn_007</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Capacitor greater than 1 MVAR</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Capacitor configured rating is greater than 1 MVAR.</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Review capacitor KVAR settings and confirm the converted model values.</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
         <is>
           <t>Dkn_00308</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="J8" t="inlineStr">
         <is>
           <t>Cap Dkn_007</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="K8" t="inlineStr">
         <is>
           <t>ABC</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="L8" t="inlineStr">
         <is>
           <t>YG</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="M8" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
+      <c r="N8" t="inlineStr">
         <is>
           <t>VOLTS</t>
         </is>
       </c>
-      <c r="G8" t="n">
-        <v>1</v>
-      </c>
-      <c r="H8" t="n">
-        <v>0</v>
-      </c>
-      <c r="I8" t="n">
+      <c r="O8" t="n">
+        <v>1</v>
+      </c>
+      <c r="P8" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q8" t="n">
         <v>600</v>
       </c>
-      <c r="J8" t="n">
+      <c r="R8" t="n">
         <v>600</v>
       </c>
-      <c r="K8" t="n">
+      <c r="S8" t="n">
         <v>600</v>
       </c>
-      <c r="L8" t="n">
-        <v>1</v>
-      </c>
-      <c r="M8" t="n">
-        <v>1</v>
-      </c>
-      <c r="N8" t="n">
+      <c r="T8" t="n">
+        <v>1</v>
+      </c>
+      <c r="U8" t="n">
+        <v>1</v>
+      </c>
+      <c r="V8" t="n">
         <v>400</v>
       </c>
-      <c r="O8" t="n">
+      <c r="W8" t="n">
         <v>119</v>
       </c>
-      <c r="P8" t="n">
+      <c r="X8" t="n">
         <v>121</v>
       </c>
-      <c r="Q8" t="n">
-        <v>0</v>
-      </c>
-      <c r="R8" t="n">
-        <v>0</v>
-      </c>
-      <c r="S8" t="n">
-        <v>0</v>
-      </c>
-      <c r="T8" t="n">
-        <v>0</v>
-      </c>
-      <c r="U8" t="n">
-        <v>0</v>
-      </c>
-      <c r="V8" t="n">
-        <v>0</v>
-      </c>
-      <c r="W8" t="n">
-        <v>0</v>
-      </c>
-      <c r="X8" t="n">
-        <v>0</v>
-      </c>
       <c r="Y8" t="n">
         <v>0</v>
       </c>
@@ -14414,202 +14372,198 @@
         <v>0</v>
       </c>
       <c r="AC8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AH8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK8" t="n">
         <v>165.833</v>
       </c>
-      <c r="AD8" t="n">
+      <c r="AL8" t="n">
         <v>120</v>
       </c>
-      <c r="AE8" t="n">
-        <v>0</v>
-      </c>
-      <c r="AF8" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG8" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH8" t="inlineStr">
+      <c r="AM8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP8" t="inlineStr">
         <is>
           <t>*</t>
         </is>
       </c>
-      <c r="AI8" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ8" t="n">
-        <v>0</v>
-      </c>
-      <c r="AK8" t="n">
-        <v>0</v>
-      </c>
-      <c r="AL8" t="n">
+      <c r="AQ8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT8" t="n">
         <v>100</v>
       </c>
-      <c r="AM8" t="inlineStr">
+      <c r="AU8" t="inlineStr">
         <is>
           <t> </t>
         </is>
       </c>
-      <c r="AN8" t="inlineStr">
+      <c r="AV8" t="inlineStr">
         <is>
           <t> </t>
         </is>
       </c>
-      <c r="AO8" t="n">
-        <v>1</v>
-      </c>
-      <c r="AP8" t="n">
+      <c r="AW8" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX8" t="n">
         <v>300</v>
       </c>
-      <c r="AQ8" t="n">
-        <v>0</v>
-      </c>
-      <c r="AR8" t="n">
+      <c r="AY8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ8" t="n">
         <v>122</v>
       </c>
-      <c r="AS8" t="n">
+      <c r="BA8" t="n">
         <v>600</v>
       </c>
-      <c r="AT8" t="n">
+      <c r="BB8" t="n">
         <v>1200</v>
       </c>
-      <c r="AU8" t="n">
+      <c r="BC8" t="n">
         <v>1200</v>
       </c>
-      <c r="AV8" t="inlineStr">
+      <c r="BD8" t="inlineStr">
         <is>
           <t> </t>
         </is>
       </c>
-      <c r="AW8" t="n">
-        <v>1</v>
-      </c>
-      <c r="AX8" t="n">
-        <v>0</v>
-      </c>
-      <c r="AY8" t="n">
-        <v>0</v>
-      </c>
-      <c r="AZ8" t="n">
+      <c r="BE8" t="n">
+        <v>1</v>
+      </c>
+      <c r="BF8" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG8" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH8" t="n">
         <v>1800</v>
       </c>
-      <c r="BA8" t="n">
+      <c r="BI8" t="n">
         <v>400</v>
       </c>
-      <c r="BB8" t="n">
+      <c r="BJ8" t="n">
         <v>2200</v>
-      </c>
-      <c r="BC8" t="inlineStr">
-        <is>
-          <t>&gt;1 MVAR</t>
-        </is>
-      </c>
-      <c r="BD8" t="inlineStr">
-        <is>
-          <t>VR5</t>
-        </is>
-      </c>
-      <c r="BE8" t="inlineStr">
-        <is>
-          <t>Component / Device</t>
-        </is>
-      </c>
-      <c r="BF8" t="inlineStr">
-        <is>
-          <t>Warning</t>
-        </is>
-      </c>
-      <c r="BG8" t="inlineStr">
-        <is>
-          <t>Capacitor</t>
-        </is>
-      </c>
-      <c r="BH8" t="inlineStr">
-        <is>
-          <t>Cap Dkn_007</t>
-        </is>
-      </c>
-      <c r="BI8" t="inlineStr">
-        <is>
-          <t>Capacitor configuration is outside expected validation limits.</t>
-        </is>
-      </c>
-      <c r="BJ8" t="inlineStr">
-        <is>
-          <t>Review capacitor KVAR settings and confirm the converted model values.</t>
-        </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" t="inlineStr"/>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Component / Device</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Warning</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Capacitor</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Cap Dkn_008</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Capacitor greater than 1 MVAR</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Capacitor configured rating is greater than 1 MVAR.</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Review capacitor KVAR settings and confirm the converted model values.</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
         <is>
           <t>Dkn_00334</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="J9" t="inlineStr">
         <is>
           <t>Cap Dkn_008</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="K9" t="inlineStr">
         <is>
           <t>ABC</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="L9" t="inlineStr">
         <is>
           <t>YG</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="M9" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
+      <c r="N9" t="inlineStr">
         <is>
           <t>PF</t>
         </is>
       </c>
-      <c r="G9" t="n">
-        <v>1</v>
-      </c>
-      <c r="H9" t="n">
-        <v>0</v>
-      </c>
-      <c r="I9" t="n">
+      <c r="O9" t="n">
+        <v>1</v>
+      </c>
+      <c r="P9" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q9" t="n">
         <v>600</v>
       </c>
-      <c r="J9" t="n">
+      <c r="R9" t="n">
         <v>600</v>
       </c>
-      <c r="K9" t="n">
+      <c r="S9" t="n">
         <v>600</v>
       </c>
-      <c r="L9" t="n">
-        <v>0</v>
-      </c>
-      <c r="M9" t="n">
-        <v>0</v>
-      </c>
-      <c r="N9" t="n">
-        <v>0</v>
-      </c>
-      <c r="O9" t="n">
-        <v>0</v>
-      </c>
-      <c r="P9" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q9" t="n">
-        <v>0</v>
-      </c>
-      <c r="R9" t="n">
-        <v>0</v>
-      </c>
-      <c r="S9" t="n">
-        <v>0</v>
-      </c>
       <c r="T9" t="n">
         <v>0</v>
       </c>
@@ -14652,188 +14606,184 @@
       <c r="AG9" t="n">
         <v>0</v>
       </c>
-      <c r="AH9" t="inlineStr">
+      <c r="AH9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP9" t="inlineStr">
         <is>
           <t>*</t>
         </is>
       </c>
-      <c r="AI9" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ9" t="n">
-        <v>0</v>
-      </c>
-      <c r="AK9" t="n">
-        <v>0</v>
-      </c>
-      <c r="AL9" t="n">
+      <c r="AQ9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT9" t="n">
         <v>100</v>
       </c>
-      <c r="AM9" t="inlineStr">
+      <c r="AU9" t="inlineStr">
         <is>
           <t> </t>
         </is>
       </c>
-      <c r="AN9" t="inlineStr">
+      <c r="AV9" t="inlineStr">
         <is>
           <t> </t>
         </is>
       </c>
-      <c r="AO9" t="n">
-        <v>1</v>
-      </c>
-      <c r="AP9" t="n">
+      <c r="AW9" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX9" t="n">
         <v>300</v>
       </c>
-      <c r="AQ9" t="n">
-        <v>0</v>
-      </c>
-      <c r="AR9" t="n">
+      <c r="AY9" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ9" t="n">
         <v>122</v>
       </c>
-      <c r="AS9" t="n">
+      <c r="BA9" t="n">
         <v>600</v>
       </c>
-      <c r="AT9" t="n">
+      <c r="BB9" t="n">
         <v>1200</v>
       </c>
-      <c r="AU9" t="n">
+      <c r="BC9" t="n">
         <v>1200</v>
       </c>
-      <c r="AV9" t="inlineStr">
+      <c r="BD9" t="inlineStr">
         <is>
           <t> </t>
         </is>
       </c>
-      <c r="AW9" t="n">
-        <v>0</v>
-      </c>
-      <c r="AX9" t="n">
-        <v>0</v>
-      </c>
-      <c r="AY9" t="n">
-        <v>0</v>
-      </c>
-      <c r="AZ9" t="n">
+      <c r="BE9" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF9" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG9" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH9" t="n">
         <v>1800</v>
       </c>
-      <c r="BA9" t="n">
-        <v>0</v>
-      </c>
-      <c r="BB9" t="n">
+      <c r="BI9" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ9" t="n">
         <v>1800</v>
-      </c>
-      <c r="BC9" t="inlineStr">
-        <is>
-          <t>&gt;1 MVAR</t>
-        </is>
-      </c>
-      <c r="BD9" t="inlineStr">
-        <is>
-          <t>VR5</t>
-        </is>
-      </c>
-      <c r="BE9" t="inlineStr">
-        <is>
-          <t>Component / Device</t>
-        </is>
-      </c>
-      <c r="BF9" t="inlineStr">
-        <is>
-          <t>Warning</t>
-        </is>
-      </c>
-      <c r="BG9" t="inlineStr">
-        <is>
-          <t>Capacitor</t>
-        </is>
-      </c>
-      <c r="BH9" t="inlineStr">
-        <is>
-          <t>Cap Dkn_008</t>
-        </is>
-      </c>
-      <c r="BI9" t="inlineStr">
-        <is>
-          <t>Capacitor configuration is outside expected validation limits.</t>
-        </is>
-      </c>
-      <c r="BJ9" t="inlineStr">
-        <is>
-          <t>Review capacitor KVAR settings and confirm the converted model values.</t>
-        </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" t="inlineStr"/>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Component / Device</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Warning</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Capacitor</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Cap Lhr_00004</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Capacitor greater than 1 MVAR</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Capacitor configured rating is greater than 1 MVAR.</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Review capacitor KVAR settings and confirm the converted model values.</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
         <is>
           <t>Lhr_00004</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="J10" t="inlineStr">
         <is>
           <t>Cap Lhr_00004</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="K10" t="inlineStr">
         <is>
           <t>ABC</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="L10" t="inlineStr">
         <is>
           <t>YG</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="M10" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
+      <c r="N10" t="inlineStr">
         <is>
           <t>PF</t>
         </is>
       </c>
-      <c r="G10" t="n">
-        <v>1</v>
-      </c>
-      <c r="H10" t="n">
-        <v>0</v>
-      </c>
-      <c r="I10" t="n">
+      <c r="O10" t="n">
+        <v>1</v>
+      </c>
+      <c r="P10" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q10" t="n">
         <v>600</v>
       </c>
-      <c r="J10" t="n">
+      <c r="R10" t="n">
         <v>600</v>
       </c>
-      <c r="K10" t="n">
+      <c r="S10" t="n">
         <v>600</v>
       </c>
-      <c r="L10" t="n">
-        <v>0</v>
-      </c>
-      <c r="M10" t="n">
-        <v>0</v>
-      </c>
-      <c r="N10" t="n">
-        <v>0</v>
-      </c>
-      <c r="O10" t="n">
-        <v>0</v>
-      </c>
-      <c r="P10" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q10" t="n">
-        <v>0</v>
-      </c>
-      <c r="R10" t="n">
-        <v>0</v>
-      </c>
-      <c r="S10" t="n">
-        <v>0</v>
-      </c>
       <c r="T10" t="n">
         <v>0</v>
       </c>
@@ -14876,188 +14826,184 @@
       <c r="AG10" t="n">
         <v>0</v>
       </c>
-      <c r="AH10" t="inlineStr">
+      <c r="AH10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP10" t="inlineStr">
         <is>
           <t>*</t>
         </is>
       </c>
-      <c r="AI10" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ10" t="n">
-        <v>0</v>
-      </c>
-      <c r="AK10" t="n">
-        <v>0</v>
-      </c>
-      <c r="AL10" t="n">
+      <c r="AQ10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT10" t="n">
         <v>100</v>
       </c>
-      <c r="AM10" t="inlineStr">
+      <c r="AU10" t="inlineStr">
         <is>
           <t> </t>
         </is>
       </c>
-      <c r="AN10" t="inlineStr">
+      <c r="AV10" t="inlineStr">
         <is>
           <t> </t>
         </is>
       </c>
-      <c r="AO10" t="n">
-        <v>1</v>
-      </c>
-      <c r="AP10" t="n">
+      <c r="AW10" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX10" t="n">
         <v>300</v>
       </c>
-      <c r="AQ10" t="n">
-        <v>0</v>
-      </c>
-      <c r="AR10" t="n">
+      <c r="AY10" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ10" t="n">
         <v>122</v>
       </c>
-      <c r="AS10" t="n">
+      <c r="BA10" t="n">
         <v>600</v>
       </c>
-      <c r="AT10" t="n">
+      <c r="BB10" t="n">
         <v>1200</v>
       </c>
-      <c r="AU10" t="n">
+      <c r="BC10" t="n">
         <v>1200</v>
       </c>
-      <c r="AV10" t="inlineStr">
+      <c r="BD10" t="inlineStr">
         <is>
           <t> </t>
         </is>
       </c>
-      <c r="AW10" t="n">
-        <v>0</v>
-      </c>
-      <c r="AX10" t="n">
-        <v>0</v>
-      </c>
-      <c r="AY10" t="n">
-        <v>0</v>
-      </c>
-      <c r="AZ10" t="n">
+      <c r="BE10" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF10" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG10" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH10" t="n">
         <v>1800</v>
       </c>
-      <c r="BA10" t="n">
-        <v>0</v>
-      </c>
-      <c r="BB10" t="n">
+      <c r="BI10" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ10" t="n">
         <v>1800</v>
-      </c>
-      <c r="BC10" t="inlineStr">
-        <is>
-          <t>&gt;1 MVAR</t>
-        </is>
-      </c>
-      <c r="BD10" t="inlineStr">
-        <is>
-          <t>VR5</t>
-        </is>
-      </c>
-      <c r="BE10" t="inlineStr">
-        <is>
-          <t>Component / Device</t>
-        </is>
-      </c>
-      <c r="BF10" t="inlineStr">
-        <is>
-          <t>Warning</t>
-        </is>
-      </c>
-      <c r="BG10" t="inlineStr">
-        <is>
-          <t>Capacitor</t>
-        </is>
-      </c>
-      <c r="BH10" t="inlineStr">
-        <is>
-          <t>Cap Lhr_00004</t>
-        </is>
-      </c>
-      <c r="BI10" t="inlineStr">
-        <is>
-          <t>Capacitor configuration is outside expected validation limits.</t>
-        </is>
-      </c>
-      <c r="BJ10" t="inlineStr">
-        <is>
-          <t>Review capacitor KVAR settings and confirm the converted model values.</t>
-        </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A11" t="inlineStr"/>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Component / Device</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Warning</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Capacitor</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Cap Pmf_001</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Capacitor greater than 1 MVAR</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Capacitor configured rating is greater than 1 MVAR.</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Review capacitor KVAR settings and confirm the converted model values.</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
         <is>
           <t>Pmf_0005</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="J11" t="inlineStr">
         <is>
           <t>Cap Pmf_001</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="K11" t="inlineStr">
         <is>
           <t>ABC</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="L11" t="inlineStr">
         <is>
           <t>YG</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
+      <c r="M11" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
+      <c r="N11" t="inlineStr">
         <is>
           <t>PF</t>
         </is>
       </c>
-      <c r="G11" t="n">
-        <v>1</v>
-      </c>
-      <c r="H11" t="n">
-        <v>0</v>
-      </c>
-      <c r="I11" t="n">
+      <c r="O11" t="n">
+        <v>1</v>
+      </c>
+      <c r="P11" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q11" t="n">
         <v>400</v>
       </c>
-      <c r="J11" t="n">
+      <c r="R11" t="n">
         <v>400</v>
       </c>
-      <c r="K11" t="n">
+      <c r="S11" t="n">
         <v>400</v>
       </c>
-      <c r="L11" t="n">
-        <v>0</v>
-      </c>
-      <c r="M11" t="n">
-        <v>0</v>
-      </c>
-      <c r="N11" t="n">
-        <v>0</v>
-      </c>
-      <c r="O11" t="n">
-        <v>0</v>
-      </c>
-      <c r="P11" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q11" t="n">
-        <v>0</v>
-      </c>
-      <c r="R11" t="n">
-        <v>0</v>
-      </c>
-      <c r="S11" t="n">
-        <v>0</v>
-      </c>
       <c r="T11" t="n">
         <v>0</v>
       </c>
@@ -15100,116 +15046,100 @@
       <c r="AG11" t="n">
         <v>0</v>
       </c>
-      <c r="AH11" t="inlineStr">
+      <c r="AH11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AK11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AL11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AN11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP11" t="inlineStr">
         <is>
           <t>*</t>
         </is>
       </c>
-      <c r="AI11" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ11" t="n">
-        <v>0</v>
-      </c>
-      <c r="AK11" t="n">
-        <v>0</v>
-      </c>
-      <c r="AL11" t="n">
+      <c r="AQ11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AS11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT11" t="n">
         <v>100</v>
       </c>
-      <c r="AM11" t="inlineStr">
+      <c r="AU11" t="inlineStr">
         <is>
           <t> </t>
         </is>
       </c>
-      <c r="AN11" t="inlineStr">
+      <c r="AV11" t="inlineStr">
         <is>
           <t> </t>
         </is>
       </c>
-      <c r="AO11" t="n">
-        <v>1</v>
-      </c>
-      <c r="AP11" t="n">
+      <c r="AW11" t="n">
+        <v>1</v>
+      </c>
+      <c r="AX11" t="n">
         <v>300</v>
       </c>
-      <c r="AQ11" t="n">
-        <v>0</v>
-      </c>
-      <c r="AR11" t="n">
+      <c r="AY11" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ11" t="n">
         <v>122</v>
       </c>
-      <c r="AS11" t="n">
+      <c r="BA11" t="n">
         <v>600</v>
-      </c>
-      <c r="AT11" t="n">
-        <v>1200</v>
-      </c>
-      <c r="AU11" t="n">
-        <v>1200</v>
-      </c>
-      <c r="AV11" t="inlineStr">
-        <is>
-          <t> </t>
-        </is>
-      </c>
-      <c r="AW11" t="n">
-        <v>0</v>
-      </c>
-      <c r="AX11" t="n">
-        <v>0</v>
-      </c>
-      <c r="AY11" t="n">
-        <v>0</v>
-      </c>
-      <c r="AZ11" t="n">
-        <v>1200</v>
-      </c>
-      <c r="BA11" t="n">
-        <v>0</v>
       </c>
       <c r="BB11" t="n">
         <v>1200</v>
       </c>
-      <c r="BC11" t="inlineStr">
-        <is>
-          <t>&gt;1 MVAR</t>
-        </is>
+      <c r="BC11" t="n">
+        <v>1200</v>
       </c>
       <c r="BD11" t="inlineStr">
         <is>
-          <t>VR5</t>
-        </is>
-      </c>
-      <c r="BE11" t="inlineStr">
-        <is>
-          <t>Component / Device</t>
-        </is>
-      </c>
-      <c r="BF11" t="inlineStr">
-        <is>
-          <t>Warning</t>
-        </is>
-      </c>
-      <c r="BG11" t="inlineStr">
-        <is>
-          <t>Capacitor</t>
-        </is>
-      </c>
-      <c r="BH11" t="inlineStr">
-        <is>
-          <t>Cap Pmf_001</t>
-        </is>
-      </c>
-      <c r="BI11" t="inlineStr">
-        <is>
-          <t>Capacitor configuration is outside expected validation limits.</t>
-        </is>
-      </c>
-      <c r="BJ11" t="inlineStr">
-        <is>
-          <t>Review capacitor KVAR settings and confirm the converted model values.</t>
-        </is>
+          <t> </t>
+        </is>
+      </c>
+      <c r="BE11" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF11" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG11" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH11" t="n">
+        <v>1200</v>
+      </c>
+      <c r="BI11" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ11" t="n">
+        <v>1200</v>
       </c>
     </row>
   </sheetData>
@@ -15223,7 +15153,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AU1"/>
+  <dimension ref="A1:AW1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15449,15 +15379,25 @@
       </c>
       <c r="AS1" t="inlineStr">
         <is>
+          <t>ElementType</t>
+        </is>
+      </c>
+      <c r="AT1" t="inlineStr">
+        <is>
+          <t>ElementID</t>
+        </is>
+      </c>
+      <c r="AU1" t="inlineStr">
+        <is>
           <t>Issue</t>
         </is>
       </c>
-      <c r="AT1" t="inlineStr">
+      <c r="AV1" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="AU1" t="inlineStr">
+      <c r="AW1" t="inlineStr">
         <is>
           <t>RecommendedAction</t>
         </is>

</xml_diff>

<commit_message>
created loads.py to fulfill VR11
</commit_message>
<xml_diff>
--- a/data/exports/synergi_validation_results.xlsx
+++ b/data/exports/synergi_validation_results.xlsx
@@ -18,6 +18,7 @@
     <sheet name="OpenFuses" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="UnfedSections" sheetId="10" state="visible" r:id="rId10"/>
     <sheet name="ConductorHeight" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="NoConnectedKVA" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -423,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -526,6 +527,16 @@
       </c>
       <c r="B10" t="n">
         <v>9</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>NoConnectedKVA</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -3963,6 +3974,87 @@
       <c r="BZ10" t="inlineStr">
         <is>
           <t>Review section height/elevation value and confirm whether the value is valid for the conductor type.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>SectionId</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>LoadRecordCount</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>SectionTotalConnectedKVA</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>SectionTotalConnectedKW</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>SectionTotalConnectedKVAR</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>RuleID</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Severity</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>ElementType</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>ElementID</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Issue</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>RecommendedAction</t>
         </is>
       </c>
     </row>

</xml_diff>